<commit_message>
Updated Description, Outcome message and validation for negative test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000253/negative/01/data/unit-test-coreid-CG0135-negative.xlsx
+++ b/rules/CORE-000253/negative/01/data/unit-test-coreid-CG0135-negative.xlsx
@@ -38,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -55,6 +55,10 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <i/>
     </font>
     <font>
@@ -66,8 +70,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -87,6 +95,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -110,14 +130,16 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,10 +482,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -487,26 +509,26 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Adverse Events</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="str">
+      <c r="A4" s="4" t="str">
         <v>dd.xpt</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>Death Details</v>
       </c>
     </row>
@@ -519,7 +541,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -541,9 +563,46 @@
         <v>Error value</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D2" s="2">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>DTHFL</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>AESDTH</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>Y</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -591,306 +650,306 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Subject Death Flag</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
         <v>10</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="6">
         <v>10</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="6">
         <v>10</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>123101</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="4" t="str">
         <v>A</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>Drug A</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>A</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>Drug A</v>
       </c>
-      <c r="H5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I5" s="2" t="str">
-        <v/>
-      </c>
-      <c r="J5" s="6" t="str">
+      <c r="H5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J5" s="4" t="str">
         <v>2005-10-13T10:15</v>
       </c>
-      <c r="K5" s="6" t="str">
+      <c r="K5" s="4" t="str">
         <v>2011-01-10</v>
       </c>
-      <c r="L5" s="6" t="str">
+      <c r="L5" s="7" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
+      <c r="A6" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B6" s="6" t="str">
+      <c r="B6" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>123102</v>
       </c>
-      <c r="D6" s="6" t="str">
+      <c r="D6" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="E6" s="6" t="str">
+      <c r="E6" s="4" t="str">
         <v>Drug B</v>
       </c>
-      <c r="F6" s="6" t="str">
+      <c r="F6" s="4" t="str">
         <v>B</v>
       </c>
-      <c r="G6" s="6" t="str">
+      <c r="G6" s="4" t="str">
         <v>Drug B</v>
       </c>
-      <c r="H6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="I6" s="2" t="str">
-        <v/>
-      </c>
-      <c r="J6" s="6" t="str">
-        <v/>
-      </c>
-      <c r="K6" s="6" t="str">
-        <v/>
-      </c>
-      <c r="L6" s="6" t="str">
+      <c r="H6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="K6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L6" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
+      <c r="A7" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B7" s="6" t="str">
+      <c r="B7" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>123103</v>
       </c>
-      <c r="D7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="6" t="str">
+      <c r="D7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="4" t="str">
         <v>SCREEN FAILURE</v>
       </c>
-      <c r="I7" s="2" t="str">
-        <v/>
-      </c>
-      <c r="J7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="K7" s="6" t="str">
-        <v/>
-      </c>
-      <c r="L7" s="6" t="str">
+      <c r="I7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="K7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L7" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
+      <c r="A8" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B8" s="6" t="str">
+      <c r="B8" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>123104</v>
       </c>
-      <c r="D8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H8" s="6" t="str">
+      <c r="D8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="E8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H8" s="4" t="str">
         <v>NOT ASSIGNED</v>
       </c>
-      <c r="I8" s="2" t="str">
-        <v/>
-      </c>
-      <c r="J8" s="6" t="str">
-        <v/>
-      </c>
-      <c r="K8" s="6" t="str">
-        <v/>
-      </c>
-      <c r="L8" s="6" t="str">
+      <c r="I8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="K8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
+      <c r="A9" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B9" s="6" t="str">
+      <c r="B9" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="4" t="str">
         <v>123105</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D9" s="4" t="str">
         <v>A</v>
       </c>
-      <c r="E9" s="6" t="str">
+      <c r="E9" s="4" t="str">
         <v>Drug A</v>
       </c>
-      <c r="F9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="G9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="H9" s="6" t="str">
+      <c r="F9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H9" s="4" t="str">
         <v>ASSIGNED, NOT TREATED</v>
       </c>
-      <c r="I9" s="2" t="str">
-        <v/>
-      </c>
-      <c r="J9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="K9" s="6" t="str">
-        <v/>
-      </c>
-      <c r="L9" s="6" t="str">
+      <c r="I9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="K9" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L9" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -935,118 +994,118 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Reported Term for the Adverse Event</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Dictionary-Derived Term</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Body System or Organ Class</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Outcome of Adverse Event</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Results in Death</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5" t="str">
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6" t="str">
         <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>AE</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>123101</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>SUDDEN CARDIAC DEATH</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>SUDDEN CARDIAC DEATH</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>CARDIOVASCULAR SYSTEM</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>FATAL</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="8" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1091,118 +1150,118 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Death Detail Assessment Short Name</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Death Detail Assessment Name</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Result or Finding as Collected</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Date/Time of Collection</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="str">
+      <c r="E4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="F4" s="5" t="str">
+      <c r="F4" s="6" t="str">
         <v>40</v>
       </c>
-      <c r="G4" s="5" t="str">
+      <c r="G4" s="6" t="str">
         <v>200</v>
       </c>
-      <c r="H4" s="5" t="str">
+      <c r="H4" s="6" t="str">
         <v>200</v>
       </c>
-      <c r="I4" s="5" t="str">
+      <c r="I4" s="6" t="str">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
+      <c r="A5" s="4" t="str">
         <v>ABC123</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>DD</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="4">
         <v>123101</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="6" t="str">
+      <c r="E5" s="4" t="str">
         <v>PRCDTH</v>
       </c>
-      <c r="F5" s="6" t="str">
+      <c r="F5" s="4" t="str">
         <v>Primary Cause of Death</v>
       </c>
-      <c r="G5" s="6" t="str">
+      <c r="G5" s="4" t="str">
         <v>SUDDEN CARDIAC DEATH</v>
       </c>
-      <c r="H5" s="6" t="str">
+      <c r="H5" s="4" t="str">
         <v>SUDDEN CARDIAC DEATH</v>
       </c>
-      <c r="I5" s="6" t="str">
+      <c r="I5" s="4" t="str">
         <v>2011-01-10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated validation for negative test case.
</commit_message>
<xml_diff>
--- a/rules/CORE-000253/negative/01/data/unit-test-coreid-CG0135-negative.xlsx
+++ b/rules/CORE-000253/negative/01/data/unit-test-coreid-CG0135-negative.xlsx
@@ -38,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -64,18 +64,13 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -83,12 +78,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -130,7 +119,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -139,7 +128,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -541,7 +529,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -564,45 +552,85 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>DTHFL</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>AESDTH</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>Y</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2" t="str">
+        <v>AETERM</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <v>SUDDEN CARDIAC DEATH</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>ae.xpt</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D5" s="2">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2" t="str">
+        <v>AESTDTC</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <v>[ABSENT]</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -653,113 +681,113 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="5" t="str">
         <v>Subject Death Flag</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
-        <v>50</v>
-      </c>
-      <c r="B4" s="6">
-        <v>50</v>
-      </c>
-      <c r="C4" s="6">
-        <v>50</v>
-      </c>
-      <c r="D4" s="6">
-        <v>50</v>
-      </c>
-      <c r="E4" s="6">
-        <v>50</v>
-      </c>
-      <c r="F4" s="6">
-        <v>50</v>
-      </c>
-      <c r="G4" s="6">
-        <v>50</v>
-      </c>
-      <c r="H4" s="6">
-        <v>50</v>
-      </c>
-      <c r="I4" s="6">
-        <v>50</v>
-      </c>
-      <c r="J4" s="6">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
+        <v>50</v>
+      </c>
+      <c r="E4" s="5">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5">
         <v>10</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>10</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5">
         <v>10</v>
       </c>
     </row>
@@ -797,7 +825,7 @@
       <c r="K5" s="4" t="str">
         <v>2011-01-10</v>
       </c>
-      <c r="L5" s="7" t="str">
+      <c r="L5" s="6" t="str">
         <v/>
       </c>
     </row>
@@ -994,89 +1022,89 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Reported Term for the Adverse Event</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Dictionary-Derived Term</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Body System or Organ Class</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Outcome of Adverse Event</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Results in Death</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
-        <v>50</v>
-      </c>
-      <c r="B4" s="6">
-        <v>50</v>
-      </c>
-      <c r="C4" s="6">
-        <v>50</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
-        <v>50</v>
-      </c>
-      <c r="F4" s="6">
-        <v>50</v>
-      </c>
-      <c r="G4" s="6">
-        <v>50</v>
-      </c>
-      <c r="H4" s="6">
-        <v>50</v>
-      </c>
-      <c r="I4" s="6" t="str">
+      <c r="E4" s="5">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="str">
         <v>5</v>
       </c>
     </row>
@@ -1093,7 +1121,7 @@
       <c r="D5" s="4">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="7" t="str">
         <v>SUDDEN CARDIAC DEATH</v>
       </c>
       <c r="F5" s="4" t="str">
@@ -1105,7 +1133,7 @@
       <c r="H5" s="4" t="str">
         <v>FATAL</v>
       </c>
-      <c r="I5" s="8" t="str">
+      <c r="I5" s="6" t="str">
         <v>Y</v>
       </c>
     </row>
@@ -1150,89 +1178,89 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Death Detail Assessment Short Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Death Detail Assessment Name</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Result or Finding as Collected</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Date/Time of Collection</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
-        <v>50</v>
-      </c>
-      <c r="B4" s="6">
-        <v>50</v>
-      </c>
-      <c r="C4" s="6">
-        <v>50</v>
-      </c>
-      <c r="D4" s="6">
+      <c r="A4" s="5">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6" t="str">
+      <c r="E4" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F4" s="5" t="str">
         <v>40</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="5" t="str">
         <v>200</v>
       </c>
-      <c r="H4" s="6" t="str">
+      <c r="H4" s="5" t="str">
         <v>200</v>
       </c>
-      <c r="I4" s="6" t="str">
+      <c r="I4" s="5" t="str">
         <v>50</v>
       </c>
     </row>

</xml_diff>